<commit_message>
commit updated leave module
</commit_message>
<xml_diff>
--- a/com.orangehrm.testing/src/test/resources/locationData.xlsx
+++ b/com.orangehrm.testing/src/test/resources/locationData.xlsx
@@ -3,19 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dhans\Desktop\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28D74971-3ADA-40E9-BB9C-2D2DB2BE04A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{6BCF79FD-76DC-410E-863C-0EAFC5D89779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11835" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
+    <workbookView xWindow="3975" yWindow="540" windowWidth="15360" windowHeight="11520" activeTab="1" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -29,12 +26,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>location</t>
   </si>
@@ -58,13 +58,49 @@
   </si>
   <si>
     <t>Nkl Office</t>
+  </si>
+  <si>
+    <t>leavetype</t>
+  </si>
+  <si>
+    <t>fromDate</t>
+  </si>
+  <si>
+    <t>toDate</t>
+  </si>
+  <si>
+    <t>partialDays</t>
+  </si>
+  <si>
+    <t>startday</t>
+  </si>
+  <si>
+    <t>comments</t>
+  </si>
+  <si>
+    <t>CAN - FMLA</t>
+  </si>
+  <si>
+    <t>Start Day Only</t>
+  </si>
+  <si>
+    <t>Half Day - Morning</t>
+  </si>
+  <si>
+    <t>personal leave</t>
+  </si>
+  <si>
+    <t>2026-05-05</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -79,6 +115,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -101,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -109,6 +151,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -127,9 +172,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -167,7 +212,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -273,7 +318,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -415,7 +460,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -457,4 +502,62 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98E7BED6-EE0C-459A-BEE2-C268FC118389}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
claim, time, buzz module excel sheet commit
</commit_message>
<xml_diff>
--- a/com.orangehrm.testing/src/test/resources/locationData.xlsx
+++ b/com.orangehrm.testing/src/test/resources/locationData.xlsx
@@ -3,38 +3,26 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dhans\Desktop\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28D74971-3ADA-40E9-BB9C-2D2DB2BE04A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{DCC42AFC-67B1-4831-86D8-729E41D1D6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11835" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Claim" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:O29"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>location</t>
   </si>
@@ -58,6 +46,12 @@
   </si>
   <si>
     <t>Nkl Office</t>
+  </si>
+  <si>
+    <t>202604210000008</t>
+  </si>
+  <si>
+    <t>reference_ID</t>
   </si>
 </sst>
 </file>
@@ -101,13 +95,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -127,9 +131,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -167,7 +171,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -273,7 +277,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -415,7 +419,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -424,9 +428,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD9B19F-E0D5-4C65-BF0F-6A7C8ADEEF5D}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -440,7 +444,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -457,4 +461,36 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BF8F3BE-CD4B-4952-ABCF-0FA9261549F8}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="4"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="5"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B3" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
commit excel error cleared
</commit_message>
<xml_diff>
--- a/com.orangehrm.testing/src/test/resources/locationData.xlsx
+++ b/com.orangehrm.testing/src/test/resources/locationData.xlsx
@@ -3,16 +3,19 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{DCC42AFC-67B1-4831-86D8-729E41D1D6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{A9A3CA4D-4DD1-40AB-8451-9669FE945EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Claim" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet5" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet4" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:O29"/>
+  <oleSize ref="A1:O4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -107,10 +110,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -478,10 +481,10 @@
       <c r="B1" s="4"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="5"/>
+      <c r="B2" s="6"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B3" s="3"/>
@@ -493,4 +496,31 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFE1AD64-96F8-4E6F-8401-3DFE37F76A73}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CF2A2DA-12C8-4F44-8AA7-5BA900D620D6}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E171AB16-2E35-454A-A0AD-FDB8049FFA7C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
commit with update excel
</commit_message>
<xml_diff>
--- a/com.orangehrm.testing/src/test/resources/locationData.xlsx
+++ b/com.orangehrm.testing/src/test/resources/locationData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{B425BB84-69A5-485F-ADED-32E760A947C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{29AA8628-B7CD-401B-8211-376186FF30F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15,19 +15,10 @@
     <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:P10"/>
+  <oleSize ref="A1:O3"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -472,9 +463,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD9B19F-E0D5-4C65-BF0F-6A7C8ADEEF5D}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -488,7 +479,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -510,17 +501,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98E7BED6-EE0C-459A-BEE2-C268FC118389}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.44140625" customWidth="1"/>
+    <col min="6" max="6" width="15.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -540,7 +531,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -568,7 +559,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BE3EE73-29F6-4035-AA8D-5DB5F44B85C7}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -577,7 +568,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2CB837A-35C3-4DE4-B714-3D682FC21D52}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -586,7 +577,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{486D74B0-56B6-4969-A411-C5E961AF7E30}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
commit with excel changes
</commit_message>
<xml_diff>
--- a/com.orangehrm.testing/src/test/resources/locationData.xlsx
+++ b/com.orangehrm.testing/src/test/resources/locationData.xlsx
@@ -3,26 +3,29 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{AEAE7CB8-6843-4EFD-B5FC-869FCBC9C9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{BBC17039-4101-46C5-A696-382666885635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Candidate Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:K14"/>
+  <oleSize ref="A1:H14"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>location</t>
   </si>
@@ -48,22 +51,40 @@
     <t>Nkl Office</t>
   </si>
   <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Last Name</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Doe</t>
-  </si>
-  <si>
-    <t>John@gmail.com</t>
+    <t>leavetype</t>
+  </si>
+  <si>
+    <t>fromDate</t>
+  </si>
+  <si>
+    <t>toDate</t>
+  </si>
+  <si>
+    <t>partialDays</t>
+  </si>
+  <si>
+    <t>startday</t>
+  </si>
+  <si>
+    <t>comments</t>
+  </si>
+  <si>
+    <t>CAN - FMLA</t>
+  </si>
+  <si>
+    <t>Start Day Only</t>
+  </si>
+  <si>
+    <t>Half Day - Morning</t>
+  </si>
+  <si>
+    <t>personal leave</t>
+  </si>
+  <si>
+    <t>2026-05-05</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
   </si>
 </sst>
 </file>
@@ -87,12 +108,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <sz val="9"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -112,11 +131,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -124,10 +142,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -477,41 +496,59 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CD4E71E-8E9D-4D28-A1C9-6CADEA80076D}">
-  <dimension ref="A1:C2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98E7BED6-EE0C-459A-BEE2-C268FC118389}">
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.54296875" customWidth="1"/>
-    <col min="2" max="2" width="9.81640625" customWidth="1"/>
-    <col min="3" max="3" width="17.36328125" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14.7265625" customWidth="1"/>
+    <col min="3" max="3" width="14.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.453125" customWidth="1"/>
+    <col min="6" max="6" width="15.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C1" t="s">
         <v>10</v>
       </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{23B05AF8-62CB-4B38-8E7A-232E4E24AC5A}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
commit with excel update
</commit_message>
<xml_diff>
--- a/com.orangehrm.testing/src/test/resources/locationData.xlsx
+++ b/com.orangehrm.testing/src/test/resources/locationData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{105DEDB1-8EAF-433E-A3E6-A8E457E1A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{B9D3C87D-D4E4-46A8-AFB5-9CCBCF94C32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15,19 +15,10 @@
     <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:N9"/>
+  <oleSize ref="A1:N5"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>

</xml_diff>

<commit_message>
commit with excel updated ...
</commit_message>
<xml_diff>
--- a/com.orangehrm.testing/src/test/resources/locationData.xlsx
+++ b/com.orangehrm.testing/src/test/resources/locationData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{B38708E7-3EF4-45D9-81E5-979B302F88F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{812F1575-1737-44B9-B449-A7C666B8C808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
     <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:N5"/>
+  <oleSize ref="A1:J5"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>

<commit_message>
chages updated with excel exchanges status
</commit_message>
<xml_diff>
--- a/com.orangehrm.testing/src/test/resources/locationData.xlsx
+++ b/com.orangehrm.testing/src/test/resources/locationData.xlsx
@@ -1,31 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{A9A3CA4D-4DD1-40AB-8451-9669FE945EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{7A23B621-39DC-435B-8371-F0D29892E85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet5" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet4" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="CandidateData" sheetId="3" r:id="rId3"/>
+    <sheet name="claim" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:O4"/>
+  <oleSize ref="A1:O11"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>location</t>
   </si>
@@ -51,17 +54,71 @@
     <t>Nkl Office</t>
   </si>
   <si>
-    <t>202604210000008</t>
+    <t>leavetype</t>
+  </si>
+  <si>
+    <t>fromDate</t>
+  </si>
+  <si>
+    <t>toDate</t>
+  </si>
+  <si>
+    <t>partialDays</t>
+  </si>
+  <si>
+    <t>startday</t>
+  </si>
+  <si>
+    <t>comments</t>
+  </si>
+  <si>
+    <t>CAN - FMLA</t>
+  </si>
+  <si>
+    <t>Start Day Only</t>
+  </si>
+  <si>
+    <t>Half Day - Morning</t>
+  </si>
+  <si>
+    <t>personal leave</t>
+  </si>
+  <si>
+    <t>2026-05-05</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Doe</t>
+  </si>
+  <si>
+    <t>john@gmail.com</t>
   </si>
   <si>
     <t>reference_ID</t>
+  </si>
+  <si>
+    <t>202604220000008</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -73,6 +130,20 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -95,10 +166,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -106,18 +178,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -467,27 +540,119 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BF8F3BE-CD4B-4952-ABCF-0FA9261549F8}">
-  <dimension ref="A1:B3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98E7BED6-EE0C-459A-BEE2-C268FC118389}">
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.44140625" customWidth="1"/>
+    <col min="6" max="6" width="15.44140625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BE3EE73-29F6-4035-AA8D-5DB5F44B85C7}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" customWidth="1"/>
+    <col min="3" max="3" width="18.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{8BB261FF-6FB9-4850-84F4-55BF6D84DCD6}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2CB837A-35C3-4DE4-B714-3D682FC21D52}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" s="4"/>
+      <c r="A1" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="7"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="6"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B3" s="3"/>
+      <c r="A2" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -498,26 +663,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFE1AD64-96F8-4E6F-8401-3DFE37F76A73}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CF2A2DA-12C8-4F44-8AA7-5BA900D620D6}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E171AB16-2E35-454A-A0AD-FDB8049FFA7C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{486D74B0-56B6-4969-A411-C5E961AF7E30}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>

</xml_diff>

<commit_message>
commit with  leave module changes
</commit_message>
<xml_diff>
--- a/com.orangehrm.testing/src/test/resources/locationData.xlsx
+++ b/com.orangehrm.testing/src/test/resources/locationData.xlsx
@@ -1,16 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DEEBIGA RK\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B3825F4-FAA9-4D18-9924-C9FD853CCC50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{065BBE46-4E18-4414-A9DC-019C56B8A1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{1CCB38A0-308E-4FBF-B53F-90078C25B8C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,6 +15,7 @@
     <sheet name="My_Info" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1:N9"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -55,9 +51,6 @@
     <t>OMR Road</t>
   </si>
   <si>
-    <t>Nkl Office</t>
-  </si>
-  <si>
     <t>leavetype</t>
   </si>
   <si>
@@ -179,6 +172,9 @@
   </si>
   <si>
     <t>QA</t>
+  </si>
+  <si>
+    <t>virat Office</t>
   </si>
 </sst>
 </file>
@@ -237,7 +233,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -255,7 +251,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -275,9 +270,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -315,7 +310,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -421,7 +416,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -563,7 +558,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -572,9 +567,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD9B19F-E0D5-4C65-BF0F-6A7C8ADEEF5D}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -588,9 +583,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -610,54 +605,54 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98E7BED6-EE0C-459A-BEE2-C268FC118389}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
-    <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.44140625" customWidth="1"/>
-    <col min="6" max="6" width="15.44140625" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>11</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>12</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="B2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>16</v>
-      </c>
-      <c r="F2" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -668,33 +663,33 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BE3EE73-29F6-4035-AA8D-5DB5F44B85C7}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" customWidth="1"/>
-    <col min="2" max="2" width="10.44140625" customWidth="1"/>
-    <col min="3" max="3" width="18.5546875" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>23</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -708,17 +703,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2CB837A-35C3-4DE4-B714-3D682FC21D52}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="7"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
         <v>26</v>
-      </c>
-      <c r="B1" s="7"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
-        <v>27</v>
       </c>
       <c r="B2" s="8"/>
     </row>
@@ -734,84 +729,84 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{486D74B0-56B6-4969-A411-C5E961AF7E30}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="C1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" t="s">
         <v>31</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" t="s">
         <v>32</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" t="s">
         <v>33</v>
       </c>
-      <c r="H1" s="9" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="B2" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="F2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="9" t="s">
+      <c r="E3" t="s">
         <v>44</v>
       </c>
-      <c r="D3" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" t="s">
         <v>45</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="G3" t="s">
         <v>46</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" t="s">
         <v>47</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>